<commit_message>
Estrategia de precios por investigacion de mercado: margenes por categoria diligenciados (joyas 70%, moda 60%, juguetes/escolar 50%, regalos 30%, bebe 25%, urbana 20%, global 25%) con redondeo a 100; temporada navidena automatica 15-nov a 6-ene suma +10pts solo en categorias de regalo; orden de categorias optimizado para conversion (joyas->juguetes->urbana primero en chips, burbujas, subnav, menu, carruseles y recomendados); ids unicos ante nombres duplicados del proveedor; migracion preciosV=2 respeta precios fijos; QA matematica exhaustiva del motor, carrito, mensaje y hoja
</commit_message>
<xml_diff>
--- a/Sublimados_Majestic_Catalogo.xlsx
+++ b/Sublimados_Majestic_Catalogo.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P88"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>OSA, cenicienta, Pinguinos, DEISY LILA, STICH</t>
+          <t>cenicienta, Pinguinos, DEISY LILA, STICH, OSA MOÑO</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/59s3cxnyzjf_1789405071463.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/e3j2zd3xf5o_1789405073203.webp</t>
         </is>
       </c>
       <c r="P38" s="2" t="n">
@@ -5360,13 +5360,13 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>930d9a47-1c0a-4813-81a5-dee51ccc96be</t>
+          <t>241d370d-0a03-4406-ad18-a9a3755f21cb</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>PIJAMA FAMILIAR NAVIDEÑA</t>
+          <t>PIJAMA NAVIDAD FAMILIAR</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -5389,7 +5389,7 @@
         <v>0</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
@@ -5398,33 +5398,33 @@
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Grinch Enojado, Reno Navidad</t>
+          <t>GRINCH ENOJADO, GRICH ENOJADO, SANTA VERDE</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>VARIEDAD DE TALLAS PARA TODA LA FAMILIA</t>
+          <t>Disponible en tallas para toda la familia</t>
         </is>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/3a06c6c2txt_1789404769078.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/uc9c3z0a2am_1791910010182.webp</t>
         </is>
       </c>
       <c r="P77" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ffc59a3f-0bbb-4c8e-8f5a-dc6478217e7e</t>
+          <t>930d9a47-1c0a-4813-81a5-dee51ccc96be</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>PIJAMAS FAMILIARES</t>
+          <t>PIJAMA NAVIDEÑA DE PAREJA</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -5437,13 +5437,17 @@
       <c r="G78" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H78" s="3" t="n"/>
-      <c r="I78" s="3" t="n"/>
+      <c r="H78" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I78" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="J78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
@@ -5452,33 +5456,29 @@
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>FAMILIA SIMPSONS, FAMILIA STICH, FAMILIA AVENGERS, FAMILIA IROMAN, FAMILIA CAPITAN AMERICA</t>
-        </is>
-      </c>
-      <c r="N78" s="2" t="inlineStr">
-        <is>
-          <t>DISPONIBLES PARA TODA LA FAMILIA</t>
-        </is>
-      </c>
+          <t>Grinch Enojado, RENO VERDE, RENO BUFANDA, SANTA CARICTURA, SANTA, RENO CUADROS</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr"/>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/iorl7i3h4x_1785715610130.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/nenu0jwquta_1789404771647.webp</t>
         </is>
       </c>
       <c r="P78" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>35feb43b-d4ee-4cd0-97a4-a6461daee102</t>
+          <t>ffc59a3f-0bbb-4c8e-8f5a-dc6478217e7e</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr"/>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>PIJAMA FAMILIAR NAVIDEÑAS</t>
+          <t>PIJAMAS FAMILIARES</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -5491,12 +5491,8 @@
       <c r="G79" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H79" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I79" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="H79" s="3" t="n"/>
+      <c r="I79" s="3" t="n"/>
       <c r="J79" s="3" t="n">
         <v>0</v>
       </c>
@@ -5510,64 +5506,56 @@
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>Grinch Enojado, Reno Nuevo, Santa y Mickey, Papá Noel reno, Santa Nieve</t>
+          <t>FAMILIA SIMPSONS, FAMILIA STICH, FAMILIA AVENGERS, FAMILIA IROMAN, FAMILIA CAPITAN AMERICA</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>DISPONIBLES EN TALLAS PARA TODA LA FAMILIA</t>
+          <t>DISPONIBLES PARA TODA LA FAMILIA</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/uo66j97t3qc_1789404070898.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/iorl7i3h4x_1785715610130.webp</t>
         </is>
       </c>
       <c r="P79" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>237051ec-4251-4654-9e91-8b031dd0ac56</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>HOM-002</t>
-        </is>
-      </c>
+          <t>35feb43b-d4ee-4cd0-97a4-a6461daee102</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>PANTALON CAMISERA PAREJA</t>
+          <t>PIJAMA FAMILIAR NAVIDEÑAS</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>pijama-pareja</t>
+          <t>familiar</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>Única</t>
-        </is>
-      </c>
+      <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="3" t="n">
-        <v>95000</v>
+        <v>3</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>75000</v>
+        <v>2</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>73000</v>
+        <v>1</v>
       </c>
       <c r="J80" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
@@ -5576,33 +5564,37 @@
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>BATMAN, STAR WARS</t>
+          <t>Grinch Enojado, Reno Nuevo, Santa y Mickey, Papá Noel reno, Santa Nieve, STICH, MICKEY, STICH ROJO, GRINCH ARBOLITO, STICH AZUL, MICKEY ROJO, MICKEY ARBOLITO, STICH BLANCO</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>TALLA UNICA SEDE HASTA UNA TALLA L COMPRENDE LA PAREJA</t>
+          <t>DISPONIBLES EN TALLAS PARA TODA LA FAMILIA</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/kyjp725ch0b_1784991424843.jpg</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/uo66j97t3qc_1789404070898.webp</t>
         </is>
       </c>
       <c r="P80" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>7dcbe20c-5963-40c3-8164-3fe454daac65</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr"/>
+          <t>237051ec-4251-4654-9e91-8b031dd0ac56</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>HOM-002</t>
+        </is>
+      </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>PIJAMA PANTALON PAREJA (Copia)</t>
+          <t>PANTALON CAMISERA PAREJA</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -5617,13 +5609,13 @@
         </is>
       </c>
       <c r="G81" s="3" t="n">
-        <v>77000</v>
+        <v>95000</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>57000</v>
+        <v>75000</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>55000</v>
+        <v>73000</v>
       </c>
       <c r="J81" s="3" t="n">
         <v>0</v>
@@ -5638,33 +5630,33 @@
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>BUGEES, VEGETA Y BULMA, PICAPIEDRAS, OSO BALENCIAGA, SIMPSOM DONA, AVENGERS, IRONAM, STICH, CAPITAN AMERICA, CAPIBARA, TOM Y JERRY, SUPERMAN</t>
+          <t>BATMAN, STAR WARS</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>TALLAS UNICA</t>
+          <t>TALLA UNICA SEDE HASTA UNA TALLA L COMPRENDE LA PAREJA</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/qxxc3xmungo_1787192967336.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/kyjp725ch0b_1784991424843.jpg</t>
         </is>
       </c>
       <c r="P81" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>89c96356-7731-47ac-bb8d-a4c4806c97c9</t>
+          <t>7dcbe20c-5963-40c3-8164-3fe454daac65</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>PIJAMA PAREJA CORTA</t>
+          <t>PIJAMA PANTALON PAREJA (Copia)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -5679,13 +5671,13 @@
         </is>
       </c>
       <c r="G82" s="3" t="n">
-        <v>66000</v>
+        <v>77000</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>46000</v>
+        <v>57000</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>44000</v>
+        <v>55000</v>
       </c>
       <c r="J82" s="3" t="n">
         <v>0</v>
@@ -5700,38 +5692,38 @@
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>SCOBBY DOOD, DONALD y DEISY, BATMAN, OSO BALENCIAGA</t>
+          <t>BUGEES, VEGETA Y BULMA, PICAPIEDRAS, OSO BALENCIAGA, SIMPSOM DONA, AVENGERS, IRONAM, STICH, CAPITAN AMERICA, CAPIBARA, TOM Y JERRY, SUPERMAN</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>TALLAS UNICAS SEDEN HASTA UNA TALLA L</t>
+          <t>TALLAS UNICA</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/k8f75qd94x_1791060978764.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/qxxc3xmungo_1787192967336.webp</t>
         </is>
       </c>
       <c r="P82" s="2" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>1badab66-f476-403e-b23d-0eee029edbb5</t>
+          <t>89c96356-7731-47ac-bb8d-a4c4806c97c9</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr"/>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>JUANITA BOLERO SUBLIMADA</t>
+          <t>PIJAMA PAREJA CORTA</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>shortiras</t>
+          <t>pijama-pareja</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
@@ -5741,13 +5733,13 @@
         </is>
       </c>
       <c r="G83" s="3" t="n">
-        <v>30000</v>
+        <v>66000</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>20000</v>
+        <v>46000</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>190000</v>
+        <v>44000</v>
       </c>
       <c r="J83" s="3" t="n">
         <v>0</v>
@@ -5762,17 +5754,17 @@
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>AVOCADO FUCSIA, GARFIELD, DEISY, OSO PANDA</t>
+          <t>SCOBBY DOOD, DONALD y DEISY, BATMAN, OSO BALENCIAGA</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>TALLA UNICA</t>
+          <t>TALLAS UNICAS SEDEN HASTA UNA TALLA L</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/so5z20eowjo_1791398900377.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/k8f75qd94x_1791060978764.webp</t>
         </is>
       </c>
       <c r="P83" s="2" t="n">
@@ -5782,13 +5774,13 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>f5e1c702-f8aa-4aa1-a440-26853e562d01</t>
+          <t>1badab66-f476-403e-b23d-0eee029edbb5</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>JUANITA BOLERO UNICOLOR</t>
+          <t>JUANITA BOLERO SUBLIMADA</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -5803,13 +5795,13 @@
         </is>
       </c>
       <c r="G84" s="3" t="n">
-        <v>27000</v>
+        <v>30000</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>17000</v>
+        <v>20000</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>16000</v>
+        <v>190000</v>
       </c>
       <c r="J84" s="3" t="n">
         <v>0</v>
@@ -5824,7 +5816,7 @@
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>FUCSIA, ROJA, BEIZ, NEGRO, ROSA, BLANCO HUESO, AZUL TURQUI</t>
+          <t>AVOCADO FUCSIA, GARFIELD, DEISY, OSO PANDA</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
@@ -5834,27 +5826,23 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/w20s9ddim4r_1791399518651.webp</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/so5z20eowjo_1791398900377.webp</t>
         </is>
       </c>
       <c r="P84" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>cc4b475f-d7d8-47bd-a3d6-73439ec7046b</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>SHD-001</t>
-        </is>
-      </c>
+          <t>f5e1c702-f8aa-4aa1-a440-26853e562d01</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>SHORT TIRA MUNDIALISTA</t>
+          <t>JUANITA BOLERO UNICOLOR</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -5865,23 +5853,23 @@
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Única, Plus, Oversize</t>
+          <t>Única</t>
         </is>
       </c>
       <c r="G85" s="3" t="n">
-        <v>25000</v>
+        <v>27000</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>15000</v>
+        <v>17000</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>14000</v>
+        <v>16000</v>
       </c>
       <c r="J85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
@@ -5890,37 +5878,37 @@
       </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>BRAZIL 2, BRAZIL, COLOMBIA 2, COLOMBIA, FRANCIA</t>
+          <t>FUCSIA, ROJA, BEIZ, NEGRO, ROSA, BLANCO HUESO, AZUL TURQUI</t>
         </is>
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>SHORT TIRA AL ESTILO MUNDIAL</t>
+          <t>TALLA UNICA</t>
         </is>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/vt26asit3lo_1784684759726.jpg</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/w20s9ddim4r_1791399518651.webp</t>
         </is>
       </c>
       <c r="P85" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ceed2bf1-60e4-41c8-a23f-372380343eea</t>
+          <t>cc4b475f-d7d8-47bd-a3d6-73439ec7046b</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>STU-001</t>
+          <t>SHD-001</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>SHORT TIRA</t>
+          <t>SHORT TIRA MUNDIALISTA</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -5931,7 +5919,7 @@
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Única</t>
+          <t>Única, Plus, Oversize</t>
         </is>
       </c>
       <c r="G86" s="3" t="n">
@@ -5947,7 +5935,7 @@
         <v>0</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
@@ -5956,64 +5944,64 @@
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>HELLO KITTY, OSO LOTSO, MICKEY, PIOLIN, KITTY OSITO, TIGERS, PINGUINOS, AVOCADO, CERDITO, CAPIBARA, CORAZONES CUADRO, BAMBI, PALETA LILA, BOB ESPONJA, CINAMORROL, MINNI FLOR, ELEFANTE, AVOCADO FUCSIA, BOB BONNY, STICH, CUTE, OSO PANDA, MAFALDA, COFFEE, PIOLIN AMARILLO, OVEJA NUVE, MY MELODDY, OSA</t>
+          <t>BRAZIL 2, BRAZIL, COLOMBIA 2, COLOMBIA, FRANCIA</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>TALLA UNICA SEDE HASTA UNA TALLA L</t>
+          <t>SHORT TIRA AL ESTILO MUNDIAL</t>
         </is>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/wq6vkaejj3f_1784922917937.jpg</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/vt26asit3lo_1784684759726.jpg</t>
         </is>
       </c>
       <c r="P86" s="2" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>76053564-24d2-4662-9825-a044ec66f57a</t>
+          <t>ceed2bf1-60e4-41c8-a23f-372380343eea</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>SHD-004</t>
+          <t>STU-001</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>SHORT CAMISA PLUS</t>
+          <t>SHORT TIRA</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>shorts</t>
+          <t>shortiras</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Plus</t>
+          <t>Única</t>
         </is>
       </c>
       <c r="G87" s="3" t="n">
-        <v>33000</v>
+        <v>25000</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>23000</v>
+        <v>15000</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>22000</v>
+        <v>14000</v>
       </c>
       <c r="J87" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
@@ -6022,37 +6010,37 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>OSO DORMILON, KOALA, JIRAFFA, PANTERA ROSA</t>
+          <t>HELLO KITTY, OSO LOTSO, MICKEY, PIOLIN, KITTY OSITO, TIGERS, PINGUINOS, AVOCADO, CERDITO, CAPIBARA, CORAZONES CUADRO, BAMBI, PALETA LILA, BOB ESPONJA, CINAMORROL, MINNI FLOR, ELEFANTE, AVOCADO FUCSIA, BOB BONNY, STICH, CUTE, OSO PANDA, MAFALDA, COFFEE, PIOLIN AMARILLO, OVEJA NUVE, MY MELODDY, OSA</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>SHORT CAMISA PLUS SEDEN HASTA UNA TALLA XL</t>
+          <t>TALLA UNICA SEDE HASTA UNA TALLA L</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/cxh01qefg3v_1784913347039.jpg</t>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/wq6vkaejj3f_1784922917937.jpg</t>
         </is>
       </c>
       <c r="P87" s="2" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>3bcb126b-7745-401c-b93d-acfd68a0fe7e</t>
+          <t>76053564-24d2-4662-9825-a044ec66f57a</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>SCD1250</t>
+          <t>SHD-004</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>SHORT CAMISA</t>
+          <t>SHORT CAMISA PLUS</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -6063,17 +6051,17 @@
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Única</t>
+          <t>Plus</t>
         </is>
       </c>
       <c r="G88" s="3" t="n">
-        <v>27000</v>
+        <v>33000</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>17000</v>
+        <v>23000</v>
       </c>
       <c r="I88" s="3" t="n">
-        <v>16000</v>
+        <v>22000</v>
       </c>
       <c r="J88" s="3" t="n">
         <v>0</v>
@@ -6088,25 +6076,91 @@
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
+          <t>OSO DORMILON, KOALA, JIRAFFA, PANTERA ROSA</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>SHORT CAMISA PLUS SEDEN HASTA UNA TALLA XL</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/cxh01qefg3v_1784913347039.jpg</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>3bcb126b-7745-401c-b93d-acfd68a0fe7e</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>SCD1250</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>SHORT CAMISA</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>shorts</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Única</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>17000</v>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>16000</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
           <t>OSO LILA, POLLITO, VAQUITA, GATICO FLOR, HELLO KITTY, CERDITO</t>
         </is>
       </c>
-      <c r="N88" s="2" t="inlineStr">
+      <c r="N89" s="2" t="inlineStr">
         <is>
           <t>TALLA UNICA SEDE HASTA UNA TALLA L.</t>
         </is>
       </c>
-      <c r="O88" s="2" t="inlineStr">
+      <c r="O89" s="2" t="inlineStr">
         <is>
           <t>https://dowbsbxvxjzjjhyqmyfr.supabase.co/storage/v1/object/public/archivos/ujg84y11p3n_1784924351434.jpg</t>
         </is>
       </c>
-      <c r="P88" s="2" t="n">
+      <c r="P89" s="2" t="n">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P88"/>
+  <autoFilter ref="A1:P89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6152,7 +6206,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
@@ -6175,7 +6229,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-13 09:42</t>
+          <t>2026-10-13 13:17</t>
         </is>
       </c>
     </row>

</xml_diff>